<commit_message>
Result on Incremental Totalizer
</commit_message>
<xml_diff>
--- a/results/2026-02-25-Maxsat/Tóm tắt kết quả.xlsx
+++ b/results/2026-02-25-Maxsat/Tóm tắt kết quả.xlsx
@@ -177,16 +177,17 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -196,10 +197,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
@@ -489,353 +489,353 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="2" t="s">
+      <c r="D1" s="11"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="3" t="s">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="7">
         <v>11763.28</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="2">
         <v>186.041</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="1">
         <v>47001.25</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="1">
         <v>22</v>
       </c>
-      <c r="G3" s="4">
-        <v>24</v>
-      </c>
-      <c r="H3" s="3">
+      <c r="G3" s="2">
+        <v>24</v>
+      </c>
+      <c r="H3" s="1">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="3" t="s">
+      <c r="A4" s="9"/>
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="1">
         <v>23035.61</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="2">
         <v>15334.3</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="7">
         <v>85001.46</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="1">
         <v>20</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="2">
         <v>21</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="7">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="3" t="s">
+      <c r="A5" s="9"/>
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>42557.14</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="1">
         <v>48736.4</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="1">
         <v>90078.45</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="2">
         <v>18</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="1">
         <v>15</v>
       </c>
-      <c r="H5" s="3">
+      <c r="H5" s="1">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="9"/>
+      <c r="B6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="6">
         <f>SUM(C3:C5)</f>
         <v>77356.03</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="4">
         <f>SUM(D3:D5)</f>
         <v>64256.741000000002</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="6">
         <f>SUM(E3:E5)</f>
         <v>222081.16000000003</v>
       </c>
-      <c r="F6" s="11">
-        <f t="shared" ref="D6:H6" si="0">SUM(F3:F5)</f>
+      <c r="F6" s="6">
+        <f t="shared" ref="F6:H6" si="0">SUM(F3:F5)</f>
         <v>60</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="3">
         <f>SUM(G3:G5)</f>
         <v>60</v>
       </c>
-      <c r="H6" s="11">
+      <c r="H6" s="6">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="7">
         <v>18.09</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="2">
         <v>9.2418309999999995</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="1">
         <v>10.46034</v>
       </c>
-      <c r="F7" s="3">
-        <v>24</v>
-      </c>
-      <c r="G7" s="3">
-        <v>24</v>
-      </c>
-      <c r="H7" s="3">
+      <c r="F7" s="1">
+        <v>24</v>
+      </c>
+      <c r="G7" s="1">
+        <v>24</v>
+      </c>
+      <c r="H7" s="1">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="3" t="s">
+      <c r="A8" s="9"/>
+      <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="1">
         <v>10491.134309999999</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="7">
         <v>15017.12</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <v>7269.5829999999996</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="1">
         <v>22</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="1">
         <v>21</v>
       </c>
-      <c r="H8" s="4">
+      <c r="H8" s="2">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="3" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="7">
         <v>11762.97784</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="1">
         <v>10400.98</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="2">
         <v>5030.67</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="1">
         <v>22</v>
       </c>
-      <c r="G9" s="3">
+      <c r="G9" s="1">
         <v>22</v>
       </c>
-      <c r="H9" s="4">
+      <c r="H9" s="2">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="13" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="6">
         <f>SUM(C7:C9)</f>
         <v>22272.202149999997</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <f t="shared" ref="D10:H10" si="1">SUM(D7:D9)</f>
         <v>25427.341830999998</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="4">
         <f>SUM(E7:E9)</f>
         <v>12310.713339999998</v>
       </c>
-      <c r="F10" s="11">
+      <c r="F10" s="6">
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="3">
         <f t="shared" si="1"/>
         <v>67</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="1">
         <v>6.3201721300000004</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="2">
         <v>6.203589</v>
       </c>
-      <c r="E11" s="3">
+      <c r="E11" s="1">
         <v>8.4396679999999993</v>
       </c>
-      <c r="F11" s="3">
-        <v>24</v>
-      </c>
-      <c r="G11" s="3">
-        <v>24</v>
-      </c>
-      <c r="H11" s="3">
+      <c r="F11" s="1">
+        <v>24</v>
+      </c>
+      <c r="G11" s="1">
+        <v>24</v>
+      </c>
+      <c r="H11" s="1">
         <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="3" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="2">
         <v>24.887712709999999</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="7">
         <v>43.055799999999998</v>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="7">
         <v>94.609719999999996</v>
       </c>
-      <c r="F12" s="3">
-        <v>24</v>
-      </c>
-      <c r="G12" s="3">
-        <v>24</v>
-      </c>
-      <c r="H12" s="3">
+      <c r="F12" s="1">
+        <v>24</v>
+      </c>
+      <c r="G12" s="1">
+        <v>24</v>
+      </c>
+      <c r="H12" s="1">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="3" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="2">
         <v>26.39</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="1">
         <v>31.024049999999999</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="1">
         <v>78.652550000000005</v>
       </c>
-      <c r="F13" s="3">
-        <v>24</v>
-      </c>
-      <c r="G13" s="3">
-        <v>24</v>
-      </c>
-      <c r="H13" s="3">
+      <c r="F13" s="1">
+        <v>24</v>
+      </c>
+      <c r="G13" s="1">
+        <v>24</v>
+      </c>
+      <c r="H13" s="1">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="9"/>
+      <c r="B14" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="4">
         <f>SUM(C11:C13)</f>
         <v>57.597884839999999</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="3">
         <f>SUM(D11:D13)</f>
         <v>80.283439000000001</v>
       </c>
-      <c r="E14" s="11">
+      <c r="E14" s="6">
         <f>SUM(E11:E13)</f>
         <v>181.70193799999998</v>
       </c>
-      <c r="F14" s="5">
-        <f t="shared" ref="D14:G14" si="2">SUM(F11:F13)</f>
+      <c r="F14" s="3">
+        <f t="shared" ref="F14" si="2">SUM(F11:F13)</f>
         <v>72</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="3">
         <f>SUM(G11:G13)</f>
         <v>72</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="3">
         <f t="shared" ref="H14" si="3">SUM(H11:H13)</f>
         <v>72</v>
       </c>

</xml_diff>